<commit_message>
Base budget on fixed pack costs, not per-gram rates
The parts are fixed packs with fixed costs, so a line costs Qty x Unit price
(columns D x K) and remaining = budget - SUMPRODUCT(D,K). Drops the Rates sheet
and the VLOOKUP/ARRAYFORMULA formula from the Apps Script, the XLSX and the
README, and keeps the budget value out of the price column so it is not counted
as a cost. Rebuilds the CSV and XLSX.
</commit_message>
<xml_diff>
--- a/bom-robu-weight-budget.xlsx
+++ b/bom-robu-weight-budget.xlsx
@@ -3,8 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
     <sheet name="BOM" sheetId="1" r:id="rId1"/>
-    <sheet name="Rates" sheetId="2" r:id="rId2"/>
-    <sheet name="Budget" sheetId="3" r:id="rId3"/>
+    <sheet name="Budget" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -1793,11 +1792,7 @@
         </is>
       </c>
       <c r="J35"/>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5000</t>
-        </is>
-      </c>
+      <c r="K35"/>
       <c r="L35" t="inlineStr">
         <is>
           <t xml:space="preserve">n/a</t>
@@ -1806,7 +1801,7 @@
       <c r="M35"/>
       <c r="N35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cell E35 = total budget</t>
+          <t xml:space="preserve">Cell E35 = total budget (kept out of the price column so it is not counted as a cost)</t>
         </is>
       </c>
     </row>
@@ -1820,192 +1815,33 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Category</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">INR per gram</t>
-        </is>
+          <t xml:space="preserve">Total budget (INR)</t>
+        </is>
+      </c>
+      <c r="B1" s="1">
+        <f>BOM!E35</f>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Buzzer</t>
+          <t xml:space="preserve">BOM cost (INR)</t>
         </is>
       </c>
       <c r="B2">
-        <v>50</v>
+        <f>SUMPRODUCT(BOM!D2:D100,BOM!K2:K100)</f>
+        <v>1362.06</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Capacitor</t>
+          <t xml:space="preserve">Remaining budget (INR)</t>
         </is>
       </c>
       <c r="B3">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Diode</t>
-        </is>
-      </c>
-      <c r="B4">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Connector</t>
-        </is>
-      </c>
-      <c r="B5">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SolderPad</t>
-        </is>
-      </c>
-      <c r="B6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MOSFET</t>
-        </is>
-      </c>
-      <c r="B7">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Resistor</t>
-        </is>
-      </c>
-      <c r="B8">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">nRF52840 (Seeed XIAO)</t>
-        </is>
-      </c>
-      <c r="B9">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Carrier PCB</t>
-        </is>
-      </c>
-      <c r="B10">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Battery</t>
-        </is>
-      </c>
-      <c r="B11">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Motor</t>
-        </is>
-      </c>
-      <c r="B12">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Propeller</t>
-        </is>
-      </c>
-      <c r="B13">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Custom part (assumed)</t>
-        </is>
-      </c>
-      <c r="B14">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;cat&gt;</t>
-        </is>
-      </c>
-      <c r="B15">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Total budget (INR)</t>
-        </is>
-      </c>
-      <c r="B1" s="1">
-        <f>BOM!E35</f>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Remaining budget (Google Sheets)</t>
-        </is>
-      </c>
-      <c r="B2">
-        <f>BOM!E35-SUMPRODUCT(BOM!G2:G100,ARRAYFORMULA(IFERROR(VLOOKUP(BOM!C2:C100,Rates!$A$2:$B$100,2,FALSE),0)))</f>
-        <v>1761</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Remaining budget (Excel)</t>
-        </is>
-      </c>
-      <c r="B3">
-        <f>BOM!E35-SUMPRODUCT(SUMIF(Rates!$A$2:$A$100,BOM!$C$2:$C$100,Rates!$B$2:$B$100),BOM!$G$2:$G$100)</f>
-        <v>1761</v>
+        <f>BOM!E35-SUMPRODUCT(BOM!D2:D100,BOM!K2:K100)</f>
+        <v>3637.94</v>
       </c>
     </row>
     <row r="4">

</xml_diff>